<commit_message>
Latest Update: 12:16pm, 19/3/2026
</commit_message>
<xml_diff>
--- a/sensor_data.xlsx
+++ b/sensor_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desktop\TRC3500\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BD391AE-F817-4BFF-8753-43741EE7C6BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46304D04-336D-4CB9-8D79-FC65A1234916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2544" yWindow="2544" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -510,37 +510,19 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2">
-        <v>60</v>
-      </c>
-      <c r="B8" s="2">
-        <v>906.67</v>
-      </c>
-      <c r="C8" s="4">
-        <v>990.67</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2">
-        <v>70</v>
-      </c>
-      <c r="B9" s="2">
-        <v>306.89999999999998</v>
-      </c>
-      <c r="C9" s="4">
-        <v>990.67</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2">
-        <v>80</v>
-      </c>
-      <c r="B10" s="2">
-        <v>536.33000000000004</v>
-      </c>
-      <c r="C10" s="4">
-        <v>504.62</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>